<commit_message>
Actualicé los datos y la explicación de la boleta
</commit_message>
<xml_diff>
--- a/SEMANA09/Excel/Boleta_Pago_Grupo_B.xlsx
+++ b/SEMANA09/Excel/Boleta_Pago_Grupo_B.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="1" r:id="R65913b46e27f4c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boleta" sheetId="2" r:id="R4b475c492804471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="Ra8ca91099e7f4b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="Rfd72f3c14b454d0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gráficos" sheetId="5" r:id="Rb5da5189c2034734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="1" r:id="Rfc9fe088278348a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boleta" sheetId="2" r:id="Ra4bc083c170a4c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="Recb80e6af3894bf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="R99b80a830a7e47df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gráficos" sheetId="5" r:id="Ra371ec20932d476f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -152,7 +152,7 @@
     <x:numFmt numFmtId="203" formatCode="0.00"/>
     <x:numFmt numFmtId="204" formatCode="&quot;S/ &quot;#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="19">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -264,8 +264,14 @@
       <x:color rgb="FF176B32"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF7F4100"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="33">
+  <x:fills count="35">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -427,8 +433,18 @@
         <x:fgColor rgb="FFDCEEDB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="16">
+  <x:borders count="19">
     <x:border>
       <x:left/>
       <x:right/>
@@ -621,11 +637,48 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFF4B183"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="207">
+  <x:cellXfs count="221">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1233,6 +1286,48 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="26" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="33" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1687,7 +1782,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bd972b933804d24"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf5e8c55b737244ab"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1717,7 +1812,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3a8a8de7ecdc4147"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6d0284ab88404278"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1747,7 +1842,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcf35b7a8a81744bc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb55e86c670b44ac0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2128,7 +2223,7 @@
         <x:v>Guía académica</x:v>
       </x:c>
       <x:c r="E12" s="65" t="str">
-        <x:v>Casos 3 y 4</x:v>
+        <x:v>Solo opción AFP Guía</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -2145,7 +2240,7 @@
         <x:v>Guía académica</x:v>
       </x:c>
       <x:c r="E13" s="65" t="str">
-        <x:v>Casos 3 y 4</x:v>
+        <x:v>Solo opción AFP Guía</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -2162,15 +2257,17 @@
         <x:v>Guía académica</x:v>
       </x:c>
       <x:c r="E14" s="65" t="str">
-        <x:v>Casos 3 y 4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="10" hidden="0" customHeight="1">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
-      <x:c r="D15" s="2"/>
-      <x:c r="E15" s="2"/>
+        <x:v>Solo opción AFP Guía</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="28" hidden="0" customHeight="1">
+      <x:c r="A15" s="218" t="str">
+        <x:v>Aclaración: 1.60% corresponde a AFP Guía y también a Prima. Si se elige Habitat, la boleta usa 1.47%.</x:v>
+      </x:c>
+      <x:c r="B15" s="219"/>
+      <x:c r="C15" s="219"/>
+      <x:c r="D15" s="219"/>
+      <x:c r="E15" s="220"/>
     </x:row>
     <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="103" t="str">
@@ -2445,9 +2542,10 @@
     <x:mergeCell ref="A4:E4"/>
     <x:mergeCell ref="A16:E16"/>
     <x:mergeCell ref="A23:E23"/>
+    <x:mergeCell ref="A15:E15"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd06a44f54a8c4137"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9c5afb439ce4a2f"/>
 </x:worksheet>
 </file>
 
@@ -2495,9 +2593,7 @@
       <x:c r="H2"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="6" t="str">
-        <x:v>Simulación académica con un profesional del área y una oferta laboral verificable.</x:v>
-      </x:c>
+      <x:c r="A3" s="6"/>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
       <x:c r="D3"/>
@@ -2569,7 +2665,7 @@
         <x:v>Días laborados</x:v>
       </x:c>
       <x:c r="B8" s="128" t="n">
-        <x:v>30</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
         <x:v>Entre 1 y 30</x:v>
@@ -2585,7 +2681,7 @@
         <x:v>¿Tiene hijos?</x:v>
       </x:c>
       <x:c r="B9" s="126" t="str">
-        <x:v>No</x:v>
+        <x:v>Sí</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
         <x:v>No / Sí</x:v>
@@ -2620,7 +2716,8 @@
         <x:v>Habitat</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>Solo si eligió AFP</x:v>
+        <x:f>IF(B10&lt;&gt;"AFP","No aplica",IF(B11="AFP Guía","Comisión académica: 1.60%",IF(B11="Habitat","Comisión Habitat: 1.47%",IF(B11="Integra","Comisión Integra: 1.55%",IF(B11="Prima","Comisión Prima: 1.60%","Comisión Profuturo: 1.69%")))))</x:f>
+        <x:v>Comisión Habitat: 1.47%</x:v>
       </x:c>
       <x:c r="D11"/>
       <x:c r="E11"/>
@@ -2633,7 +2730,7 @@
         <x:v>Horas extras al 25%</x:v>
       </x:c>
       <x:c r="B12" s="129" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>Mayor o igual a cero</x:v>
@@ -2649,7 +2746,7 @@
         <x:v>Horas extras al 35%</x:v>
       </x:c>
       <x:c r="B13" s="129" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Mayor o igual a cero</x:v>
@@ -2665,7 +2762,7 @@
         <x:v>Adelantos</x:v>
       </x:c>
       <x:c r="B14" s="196" t="n">
-        <x:v>0</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
         <x:v>Mayor o igual a cero</x:v>
@@ -2786,7 +2883,7 @@
       </x:c>
       <x:c r="B23" s="197" t="n">
         <x:f>ROUND($B$7/30*$B$8,2)</x:f>
-        <x:v>4000</x:v>
+        <x:v>3466.67</x:v>
       </x:c>
       <x:c r="C23" s="2"/>
       <x:c r="D23"/>
@@ -2801,7 +2898,7 @@
       </x:c>
       <x:c r="B24" s="197" t="n">
         <x:f>IF($B$9="Sí",ROUND('Parámetros'!$B$6*'Parámetros'!$B$7,2),0)</x:f>
-        <x:v>0</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C24" s="2"/>
       <x:c r="D24"/>
@@ -2816,7 +2913,7 @@
       </x:c>
       <x:c r="B25" s="197" t="n">
         <x:f>ROUND(($B$7/30/8)*(1+'Parámetros'!$B$10)*$B$12,2)</x:f>
-        <x:v>0</x:v>
+        <x:v>41.67</x:v>
       </x:c>
       <x:c r="C25" s="2"/>
       <x:c r="D25"/>
@@ -2831,7 +2928,7 @@
       </x:c>
       <x:c r="B26" s="197" t="n">
         <x:f>ROUND(($B$7/30/8)*(1+'Parámetros'!$B$11)*$B$13,2)</x:f>
-        <x:v>0</x:v>
+        <x:v>67.5</x:v>
       </x:c>
       <x:c r="C26" s="2"/>
       <x:c r="D26"/>
@@ -2846,7 +2943,7 @@
       </x:c>
       <x:c r="B27" s="198" t="n">
         <x:f>ROUND(SUM(B23:B26),2)</x:f>
-        <x:v>4000</x:v>
+        <x:v>3698.84</x:v>
       </x:c>
       <x:c r="C27" s="2"/>
       <x:c r="D27"/>
@@ -2914,7 +3011,7 @@
       </x:c>
       <x:c r="B32" s="197" t="n">
         <x:f>IF($B$10="AFP",ROUND($B$27*IF($B$11="AFP Guía",'Parámetros'!$B$12,0.10),2),0)</x:f>
-        <x:v>400</x:v>
+        <x:v>369.88</x:v>
       </x:c>
       <x:c r="C32" s="2"/>
       <x:c r="D32"/>
@@ -2929,7 +3026,7 @@
       </x:c>
       <x:c r="B33" s="197" t="n">
         <x:f>IF($B$10="AFP",ROUND($B$27*IF($B$11="AFP Guía",'Parámetros'!$B$13,IF($B$11="Habitat",'Parámetros'!$C$18,IF($B$11="Integra",'Parámetros'!$C$19,IF($B$11="Prima",'Parámetros'!$C$20,'Parámetros'!$C$21)))),2),0)</x:f>
-        <x:v>58.8</x:v>
+        <x:v>54.37</x:v>
       </x:c>
       <x:c r="C33" s="2"/>
       <x:c r="D33"/>
@@ -2944,7 +3041,7 @@
       </x:c>
       <x:c r="B34" s="197" t="n">
         <x:f>IF($B$10="AFP",ROUND($B$27*IF($B$11="AFP Guía",'Parámetros'!$B$14,'Parámetros'!$D$18),2),0)</x:f>
-        <x:v>54.8</x:v>
+        <x:v>50.67</x:v>
       </x:c>
       <x:c r="C34" s="2"/>
       <x:c r="D34"/>
@@ -2959,7 +3056,7 @@
       </x:c>
       <x:c r="B35" s="197" t="n">
         <x:f>ROUND($B$14,2)</x:f>
-        <x:v>0</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C35" s="2"/>
       <x:c r="D35"/>
@@ -2974,7 +3071,7 @@
       </x:c>
       <x:c r="B36" s="198" t="n">
         <x:f>ROUND(SUM(B31:B35),2)</x:f>
-        <x:v>513.6</x:v>
+        <x:v>624.92</x:v>
       </x:c>
       <x:c r="C36"/>
       <x:c r="D36"/>
@@ -3027,7 +3124,7 @@
       </x:c>
       <x:c r="B40" s="197" t="n">
         <x:f>ROUND($B$27*'Parámetros'!$B$9,2)</x:f>
-        <x:v>360</x:v>
+        <x:v>332.9</x:v>
       </x:c>
       <x:c r="C40" s="2"/>
     </x:row>
@@ -3037,7 +3134,7 @@
       </x:c>
       <x:c r="B41" s="205" t="n">
         <x:f>ROUND(B27+B40,2)</x:f>
-        <x:v>4360</x:v>
+        <x:v>4031.74</x:v>
       </x:c>
       <x:c r="C41" s="2"/>
     </x:row>
@@ -3053,7 +3150,7 @@
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="140" t="n">
         <x:f>ROUND($B$27-$B$36,2)</x:f>
-        <x:v>3486.4</x:v>
+        <x:v>3073.92</x:v>
       </x:c>
       <x:c r="B43" s="140"/>
       <x:c r="C43" s="2"/>
@@ -3105,7 +3202,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de4d4a15b624a46"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89dd1d8934b84863"/>
 </x:worksheet>
 </file>
 
@@ -5680,7 +5777,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf8cea55787346f0"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a30004a27c247b3"/>
 </x:worksheet>
 </file>
 
@@ -5906,11 +6003,13 @@
         <x:v>292.77</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="10" hidden="0" customHeight="1">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
+    <x:row r="17" ht="30" hidden="0" customHeight="1">
+      <x:c r="A17" s="218" t="str">
+        <x:v>Comisión AFP: se usa la tasa de la AFP elegida. Habitat 1.47%, Integra 1.55%, Prima 1.60% y Profuturo 1.69%. El 1.60% de AFP Guía se reserva para los casos académicos.</x:v>
+      </x:c>
+      <x:c r="B17" s="219"/>
+      <x:c r="C17" s="219"/>
+      <x:c r="D17" s="220"/>
     </x:row>
     <x:row r="18" ht="10" hidden="0" customHeight="1">
       <x:c r="A18" s="2"/>
@@ -6089,6 +6188,7 @@
     <x:mergeCell ref="A4:D4"/>
     <x:mergeCell ref="A19:D19"/>
     <x:mergeCell ref="A28:D28"/>
+    <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7272,6 +7372,6 @@
     <x:mergeCell ref="A42:L42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d471f371b7941d0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5948598325a64cf0"/>
 </x:worksheet>
 </file>
</xml_diff>